<commit_message>
Hojas de encargo de Drive: 2022
Leidas las firmadas sin enviada (algunas son correos de FAIN con el
encargo o los codigos de pedido: a facturacion). Regla: el 'inicio de
obra' con precio es un hito de la DF.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cruce_hojas_2023.xlsx
+++ b/docs/cruce_hojas_2023.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -79,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -94,9 +89,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4519,14 +4511,14 @@
           <t>Y23_044</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: Informe pericial (RABAT 10): cobra 300 € de 'gastos colegiales' (visado) en línea aparte. ¿Qué bloque? ¿O va dentro del informe?</t>
+          <t>RESUELTO LEYENDO: Los gastos de visado NUNCA se cobran (Mónica): aquí se cobraron 300 € como excepción escrita a mano en la hoja; van como línea del informe, comentada.</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -4558,7 +4550,7 @@
       <c r="J48" s="2" t="inlineStr">
         <is>
           <t>TOMA DE DATOS Y MODELADO 3D: 400 €
-SIN CASAR: 300 €
+INFORME PERICIAL: 300 €
 INFORME PERICIAL: 2000 €
 TRAMITACION LICENCIAS: incluido
 DF: 400 €</t>
@@ -10794,12 +10786,12 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Gastos colegiales</t>
+          <t>Gastos colegiales (visado) — excepción escrita a mano</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>SIN CASAR</t>
+          <t>INFORME PERICIAL</t>
         </is>
       </c>
       <c r="E156" s="2" t="n">

</xml_diff>